<commit_message>
fix distancias y velocidades
</commit_message>
<xml_diff>
--- a/docs/configuraciones.xlsx
+++ b/docs/configuraciones.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanapolsky\GoogleDriveSA\Python 2.0\github\Urbantrips_new\mendoza\UrbanTrips\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanapolsky\GoogleDriveSA\Python 2.0\github\Urbantrips_new\urbantrips_2026\UrbanTrips\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2DCB6C-4C93-4283-A844-04279210D688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EF0B5A-2E44-44C4-A798-B645E7CDFA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="164">
   <si>
     <t>orden</t>
   </si>
@@ -511,6 +511,12 @@
   </si>
   <si>
     <t>distance_servicio_mts_agg_gps</t>
+  </si>
+  <si>
+    <t>dominio_gps</t>
+  </si>
+  <si>
+    <t>Dominio o Mounting kit del vehículo</t>
   </si>
 </sst>
 </file>
@@ -855,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1619,150 +1625,154 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>3.1</v>
+        <v>2.94</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>11</v>
+        <v>86</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>162</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>101</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J43" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="J44" s="4"/>
+        <v>102</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F45" s="3">
-        <v>5</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>82</v>
+        <v>106</v>
+      </c>
+      <c r="F46" s="3">
+        <v>5</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>110</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J47" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C48" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>3.7</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H48" s="3" t="s">
+      <c r="H49" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="J48" s="4"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
         <v>4.0999999999999996</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>4.2</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>115</v>
@@ -1771,12 +1781,12 @@
         <v>115</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>115</v>
@@ -1785,12 +1795,12 @@
         <v>115</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>4.4000000000000004</v>
+        <v>4.3</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>115</v>
@@ -1799,12 +1809,12 @@
         <v>115</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>4.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>115</v>
@@ -1813,12 +1823,12 @@
         <v>115</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>4.5999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>115</v>
@@ -1827,12 +1837,12 @@
         <v>115</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>115</v>
@@ -1841,12 +1851,12 @@
         <v>115</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>115</v>
@@ -1855,43 +1865,43 @@
         <v>115</v>
       </c>
       <c r="D56" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D57" s="3" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
         <v>5.0999999999999996</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B58" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C58" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H57" s="3" t="s">
+      <c r="H58" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="I57" s="3" t="s">
+      <c r="I58" s="3" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
         <v>5.2</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
-        <v>5.3</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>128</v>
@@ -1900,12 +1910,12 @@
         <v>129</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>128</v>
@@ -1914,12 +1924,12 @@
         <v>129</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>128</v>
@@ -1928,57 +1938,57 @@
         <v>129</v>
       </c>
       <c r="D61" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D62" s="3" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
         <v>6.1</v>
       </c>
-      <c r="B62" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D62" s="3" t="s">
+      <c r="B63" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D63" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="I62" s="3" t="s">
+      <c r="I63" s="3" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
         <v>6.2</v>
       </c>
-      <c r="B63" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D63" s="3" t="s">
+      <c r="B64" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D64" s="3" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>134</v>
@@ -1987,12 +1997,12 @@
         <v>134</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>134</v>
@@ -2001,12 +2011,12 @@
         <v>134</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>134</v>
@@ -2015,12 +2025,12 @@
         <v>134</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>134</v>
@@ -2029,12 +2039,12 @@
         <v>134</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>134</v>
@@ -2043,12 +2053,12 @@
         <v>134</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>134</v>
@@ -2057,12 +2067,12 @@
         <v>134</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>134</v>
@@ -2071,12 +2081,12 @@
         <v>134</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>134</v>
@@ -2085,12 +2095,12 @@
         <v>134</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>134</v>
@@ -2099,12 +2109,12 @@
         <v>134</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>134</v>
@@ -2113,12 +2123,12 @@
         <v>134</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>134</v>
@@ -2127,12 +2137,12 @@
         <v>134</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>134</v>
@@ -2141,37 +2151,51 @@
         <v>134</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>152</v>
+        <v>134</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
         <v>9.1</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B79" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C79" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H78" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>154</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add batches to config
</commit_message>
<xml_diff>
--- a/docs/configuraciones.xlsx
+++ b/docs/configuraciones.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanapolsky\GoogleDriveSA\Python 2.0\github\Urbantrips_new\urbantrips_2026\UrbanTrips\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanapolsky\urbantrips_sin_drive\urbantrips_refactor\UrbanTrips\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EF0B5A-2E44-44C4-A798-B645E7CDFA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940109D3-AF37-4B45-8B39-6F43D1FE12E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="166">
   <si>
     <t>orden</t>
   </si>
@@ -517,6 +517,12 @@
   </si>
   <si>
     <t>Dominio o Mounting kit del vehículo</t>
+  </si>
+  <si>
+    <t>n_batches</t>
+  </si>
+  <si>
+    <t>traveler partitions; controls memory per processing batch</t>
   </si>
 </sst>
 </file>
@@ -861,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1260,177 +1266,173 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>2.44</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>11</v>
+        <v>164</v>
+      </c>
+      <c r="F21" s="3">
+        <v>30</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>60</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>2.4500000000000002</v>
+        <v>2.44</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G22" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>2.46</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>11</v>
+        <v>62</v>
+      </c>
+      <c r="F23" s="3">
+        <v>2000</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>2.5</v>
+        <v>2.46</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" s="3">
-        <v>8</v>
+        <v>65</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>2.5099999999999998</v>
+        <v>2.5</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F25" s="3">
-        <v>9265</v>
+        <v>8</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>2.6</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="F26" s="3">
+        <v>9265</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>2.71</v>
+        <v>2.61</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="J28" s="1"/>
+        <v>78</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>2.7</v>
+        <v>2.71</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>82</v>
@@ -1438,27 +1440,31 @@
       <c r="G29" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="H29" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="J29" s="1"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>85</v>
@@ -1467,12 +1473,15 @@
         <v>86</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>2.82</v>
+        <v>2.81</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>85</v>
@@ -1481,12 +1490,12 @@
         <v>86</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>2.83</v>
+        <v>2.82</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>85</v>
@@ -1495,12 +1504,12 @@
         <v>86</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>85</v>
@@ -1509,12 +1518,12 @@
         <v>86</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>85</v>
@@ -1523,12 +1532,12 @@
         <v>86</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>2.86</v>
+        <v>2.85</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>85</v>
@@ -1537,12 +1546,12 @@
         <v>86</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>2.88</v>
+        <v>2.86</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>85</v>
@@ -1551,12 +1560,12 @@
         <v>86</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>2.89</v>
+        <v>2.88</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>85</v>
@@ -1565,15 +1574,12 @@
         <v>86</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>156</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>2.91</v>
+        <v>2.89</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>85</v>
@@ -1582,15 +1588,15 @@
         <v>86</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>85</v>
@@ -1599,15 +1605,15 @@
         <v>86</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>85</v>
@@ -1616,16 +1622,15 @@
         <v>86</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J41" s="4"/>
+        <v>159</v>
+      </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>2.94</v>
+        <v>2.93</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>85</v>
@@ -1634,159 +1639,163 @@
         <v>86</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>163</v>
+        <v>97</v>
       </c>
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>3.1</v>
+        <v>2.94</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>11</v>
+        <v>86</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>162</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>101</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="J43" s="4"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="J45" s="4"/>
+        <v>102</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F46" s="3">
-        <v>5</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>82</v>
+        <v>106</v>
+      </c>
+      <c r="F47" s="3">
+        <v>5</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="I47" s="3" t="s">
-        <v>110</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J48" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>4.0999999999999996</v>
+        <v>3.7</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>116</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>115</v>
@@ -1795,12 +1804,12 @@
         <v>115</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>115</v>
@@ -1809,12 +1818,12 @@
         <v>115</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>4.4000000000000004</v>
+        <v>4.3</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>115</v>
@@ -1823,12 +1832,12 @@
         <v>115</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>4.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>115</v>
@@ -1837,12 +1846,12 @@
         <v>115</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>4.5999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>115</v>
@@ -1851,12 +1860,12 @@
         <v>115</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>115</v>
@@ -1865,12 +1874,12 @@
         <v>115</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>115</v>
@@ -1879,43 +1888,43 @@
         <v>115</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>128</v>
@@ -1924,12 +1933,12 @@
         <v>129</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>128</v>
@@ -1938,12 +1947,12 @@
         <v>129</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>128</v>
@@ -1952,29 +1961,26 @@
         <v>129</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>6.1</v>
+        <v>5.5</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>134</v>
@@ -1983,12 +1989,15 @@
         <v>134</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>134</v>
@@ -1997,12 +2006,12 @@
         <v>134</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>134</v>
@@ -2011,12 +2020,12 @@
         <v>134</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>134</v>
@@ -2025,12 +2034,12 @@
         <v>134</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>134</v>
@@ -2039,12 +2048,12 @@
         <v>134</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>134</v>
@@ -2053,12 +2062,12 @@
         <v>134</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>134</v>
@@ -2067,12 +2076,12 @@
         <v>134</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>134</v>
@@ -2081,12 +2090,12 @@
         <v>134</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>134</v>
@@ -2095,12 +2104,12 @@
         <v>134</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>134</v>
@@ -2109,12 +2118,12 @@
         <v>134</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>134</v>
@@ -2123,12 +2132,12 @@
         <v>134</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>134</v>
@@ -2137,12 +2146,12 @@
         <v>134</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>134</v>
@@ -2151,12 +2160,12 @@
         <v>134</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>134</v>
@@ -2165,37 +2174,51 @@
         <v>134</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>152</v>
+        <v>134</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
         <v>9.1</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B80" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C80" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H79" s="3" t="s">
+      <c r="H80" s="3" t="s">
         <v>154</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ubicación parametrizable de archivos temporales
</commit_message>
<xml_diff>
--- a/docs/configuraciones.xlsx
+++ b/docs/configuraciones.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sanapolsky\urbantrips_sin_drive\urbantrips_refactor\UrbanTrips\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2860BC-77C3-4EC7-A6A6-8C09F2BC3793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B49F657-86F3-456F-89CA-BEE149498537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="186">
   <si>
     <t>orden</t>
   </si>
@@ -574,6 +574,15 @@
   </si>
   <si>
     <t>Nombre de Ciudad o area Metropolitana (necesario para crear directorio de datos en matrices de distancia)</t>
+  </si>
+  <si>
+    <t>tmp_dir</t>
+  </si>
+  <si>
+    <t>Directorios temporales (opcionales; en blanco = default). Absolutos o relativos a este archivo. Funcionan igual en Windows y Linux</t>
+  </si>
+  <si>
+    <t>directorio para TODOS los archivos temporales (spill de DuckDB y staging parquet). En blanco = temp del sistema. Puede apuntar a otro disco, ej. "D:/urbantrips_tmp" o "/mnt/scratch/urbantrips"</t>
   </si>
 </sst>
 </file>
@@ -918,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1027,27 +1036,27 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>2.0099999999999998</v>
+        <v>1.6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>183</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
+        <v>183</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>20</v>
+        <v>185</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>2.02</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>16</v>
@@ -1056,18 +1065,18 @@
         <v>17</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>2.0299999999999998</v>
+        <v>2.02</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>16</v>
@@ -1076,18 +1085,18 @@
         <v>17</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>2.04</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>16</v>
@@ -1096,15 +1105,18 @@
         <v>17</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>2.0499999999999998</v>
+        <v>2.04</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>16</v>
@@ -1113,15 +1125,15 @@
         <v>17</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>2.06</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>16</v>
@@ -1130,18 +1142,15 @@
         <v>17</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>2.0699999999999998</v>
+        <v>2.06</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>16</v>
@@ -1150,15 +1159,18 @@
         <v>17</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>2.08</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>16</v>
@@ -1167,15 +1179,15 @@
         <v>17</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>2.09</v>
+        <v>2.08</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>16</v>
@@ -1184,15 +1196,15 @@
         <v>17</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>16</v>
@@ -1201,15 +1213,15 @@
         <v>17</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>2.11</v>
+        <v>2.1</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>16</v>
@@ -1218,15 +1230,15 @@
         <v>17</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>16</v>
@@ -1235,15 +1247,15 @@
         <v>17</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>2.13</v>
+        <v>2.12</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>16</v>
@@ -1252,15 +1264,15 @@
         <v>17</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>16</v>
@@ -1269,299 +1281,295 @@
         <v>17</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>2.21</v>
+        <v>2.14</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>11</v>
+        <v>17</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>2.2200000000000002</v>
+        <v>2.21</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="3">
-        <v>120</v>
+        <v>48</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>2.23</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F21" s="3">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>2.2400000000000002</v>
+        <v>2.23</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>164</v>
+        <v>54</v>
       </c>
       <c r="F22" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>165</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>2.44</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>11</v>
+        <v>164</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>60</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>2.4500000000000002</v>
+        <v>2.44</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="F24" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>2.46</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>11</v>
+        <v>62</v>
+      </c>
+      <c r="F25" s="3">
+        <v>2000</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>2.4700000000000002</v>
+        <v>2.46</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="F26" s="3">
-        <v>0.25</v>
+        <v>65</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>179</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>2.48</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F27" s="3">
-        <v>600</v>
+        <v>0.25</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>68</v>
+        <v>177</v>
       </c>
       <c r="F28" s="3">
-        <v>8</v>
+        <v>600</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>70</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>2.5099999999999998</v>
+        <v>2.5</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F29" s="3">
-        <v>9265</v>
+        <v>8</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>2.6</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="F30" s="3">
+        <v>9265</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>2.71</v>
+        <v>2.61</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="J32" s="1"/>
+        <v>78</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>2.7</v>
+        <v>2.71</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>82</v>
@@ -1569,27 +1577,31 @@
       <c r="G33" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="H33" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="J33" s="1"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>85</v>
@@ -1598,12 +1610,15 @@
         <v>86</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>2.82</v>
+        <v>2.81</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>85</v>
@@ -1612,12 +1627,12 @@
         <v>86</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>2.83</v>
+        <v>2.82</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>85</v>
@@ -1626,12 +1641,12 @@
         <v>86</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>85</v>
@@ -1640,12 +1655,12 @@
         <v>86</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>85</v>
@@ -1654,12 +1669,12 @@
         <v>86</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>2.86</v>
+        <v>2.85</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>85</v>
@@ -1668,12 +1683,12 @@
         <v>86</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>2.88</v>
+        <v>2.86</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>85</v>
@@ -1682,12 +1697,12 @@
         <v>86</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>2.89</v>
+        <v>2.88</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>85</v>
@@ -1696,15 +1711,12 @@
         <v>86</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>156</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>2.91</v>
+        <v>2.89</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>85</v>
@@ -1713,15 +1725,15 @@
         <v>86</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>85</v>
@@ -1730,15 +1742,15 @@
         <v>86</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>2.93</v>
+        <v>2.92</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>85</v>
@@ -1747,16 +1759,15 @@
         <v>86</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J45" s="4"/>
+        <v>159</v>
+      </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>2.94</v>
+        <v>2.93</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>85</v>
@@ -1765,159 +1776,163 @@
         <v>86</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>163</v>
+        <v>97</v>
       </c>
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>3.1</v>
+        <v>2.94</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>11</v>
+        <v>86</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>162</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I47" s="3" t="s">
-        <v>101</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="J49" s="4"/>
+        <v>102</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F50" s="3">
-        <v>5</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F51" s="3" t="s">
-        <v>82</v>
+        <v>106</v>
+      </c>
+      <c r="F51" s="3">
+        <v>5</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>11</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="I51" s="3" t="s">
-        <v>110</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="J51" s="4"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J52" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>96</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>4.0999999999999996</v>
+        <v>3.7</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>116</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J54" s="4"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>115</v>
@@ -1926,12 +1941,12 @@
         <v>115</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>115</v>
@@ -1940,12 +1955,12 @@
         <v>115</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>4.4000000000000004</v>
+        <v>4.3</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>115</v>
@@ -1954,12 +1969,12 @@
         <v>115</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>4.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>115</v>
@@ -1968,12 +1983,12 @@
         <v>115</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>4.5999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>115</v>
@@ -1982,12 +1997,12 @@
         <v>115</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>115</v>
@@ -1996,12 +2011,12 @@
         <v>115</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>115</v>
@@ -2010,35 +2025,26 @@
         <v>115</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>175</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>166</v>
@@ -2047,7 +2053,7 @@
         <v>166</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>82</v>
@@ -2061,7 +2067,7 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>166</v>
@@ -2070,7 +2076,7 @@
         <v>166</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>82</v>
@@ -2084,7 +2090,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>166</v>
@@ -2093,7 +2099,7 @@
         <v>166</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>82</v>
@@ -2107,7 +2113,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>166</v>
@@ -2116,7 +2122,7 @@
         <v>166</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>82</v>
@@ -2130,7 +2136,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>166</v>
@@ -2139,7 +2145,7 @@
         <v>166</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>82</v>
@@ -2153,7 +2159,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>166</v>
@@ -2162,7 +2168,7 @@
         <v>166</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F68" s="3" t="s">
         <v>82</v>
@@ -2176,7 +2182,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>166</v>
@@ -2185,7 +2191,7 @@
         <v>166</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>82</v>
@@ -2199,38 +2205,47 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>124</v>
+        <v>166</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>125</v>
+        <v>166</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>128</v>
@@ -2239,12 +2254,12 @@
         <v>129</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>128</v>
@@ -2253,12 +2268,12 @@
         <v>129</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>128</v>
@@ -2267,29 +2282,26 @@
         <v>129</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>134</v>
@@ -2298,12 +2310,15 @@
         <v>134</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>134</v>
@@ -2312,12 +2327,12 @@
         <v>134</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>134</v>
@@ -2326,12 +2341,12 @@
         <v>134</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>134</v>
@@ -2340,12 +2355,12 @@
         <v>134</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>134</v>
@@ -2354,12 +2369,12 @@
         <v>134</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>134</v>
@@ -2368,12 +2383,12 @@
         <v>134</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>134</v>
@@ -2382,12 +2397,12 @@
         <v>134</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>134</v>
@@ -2396,12 +2411,12 @@
         <v>134</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>134</v>
@@ -2410,12 +2425,12 @@
         <v>134</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>8.1999999999999993</v>
+        <v>8.1</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>134</v>
@@ -2424,12 +2439,12 @@
         <v>134</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>8.3000000000000007</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>134</v>
@@ -2438,12 +2453,12 @@
         <v>134</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>8.4</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>134</v>
@@ -2452,12 +2467,12 @@
         <v>134</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>134</v>
@@ -2466,12 +2481,12 @@
         <v>134</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>134</v>
@@ -2480,37 +2495,51 @@
         <v>134</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G90" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H90" s="3" t="s">
-        <v>152</v>
+        <v>134</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
         <v>9.1999999999999993</v>
       </c>
-      <c r="B91" s="3" t="s">
+      <c r="B92" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="C92" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H91" s="3" t="s">
+      <c r="H92" s="3" t="s">
         <v>154</v>
       </c>
     </row>

</xml_diff>